<commit_message>
Consolidate site content sources
</commit_message>
<xml_diff>
--- a/frontend/data-source/members.xlsx
+++ b/frontend/data-source/members.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教师" sheetId="1" r:id="R839197e19e2d4ea3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="博士研究生" sheetId="2" r:id="R4f79ce9782244932"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="硕士研究生" sheetId="3" r:id="R9d0a1406f8744503"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教师" sheetId="1" r:id="R886c1acdc7984091"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="博士研究生" sheetId="2" r:id="R918779fff5634bf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="硕士研究生" sheetId="3" r:id="R8ba10ab65a014773"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作者别名" sheetId="4" r:id="R721f9324300e4ed8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43,12 +44,17 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4F1670"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -75,7 +81,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -107,6 +113,11 @@
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -150,6 +161,16 @@
     <x:tableColumn id="3" name="member_type"/>
     <x:tableColumn id="4" name="identity"/>
     <x:tableColumn id="5" name="homepage"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="MemberAliasesTable" displayName="MemberAliasesTable" ref="A1:B29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="2">
+    <x:tableColumn id="1" name="alias"/>
+    <x:tableColumn id="2" name="member_id"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -352,7 +373,7 @@
   <x:cols>
     <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
@@ -390,7 +411,7 @@
         <x:v>陈振宇</x:v>
       </x:c>
       <x:c r="C2" s="11" t="str">
-        <x:v>avatar.jpg</x:v>
+        <x:v>members/teacher-001/avatar.jpg</x:v>
       </x:c>
       <x:c r="D2" s="11" t="str">
         <x:v>teacher</x:v>
@@ -413,7 +434,7 @@
         <x:v>刘嘉</x:v>
       </x:c>
       <x:c r="C3" s="12" t="str">
-        <x:v>avatar.jpg</x:v>
+        <x:v>members/teacher-002/avatar.jpg</x:v>
       </x:c>
       <x:c r="D3" s="12" t="str">
         <x:v>teacher</x:v>
@@ -436,7 +457,7 @@
         <x:v>赵志宏</x:v>
       </x:c>
       <x:c r="C4" s="12" t="str">
-        <x:v>avatar.jfif</x:v>
+        <x:v>members/teacher-003/avatar.jfif</x:v>
       </x:c>
       <x:c r="D4" s="12" t="str">
         <x:v>teacher</x:v>
@@ -457,7 +478,7 @@
         <x:v>房春荣</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>avatar.jpeg</x:v>
+        <x:v>members/teacher-004/avatar.jpeg</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
         <x:v>teacher</x:v>
@@ -480,7 +501,7 @@
         <x:v>何铁科</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>avatar.jpg</x:v>
+        <x:v>members/teacher-005/avatar.jpg</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
         <x:v>teacher</x:v>
@@ -501,7 +522,7 @@
         <x:v>王兴亚</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>avatar.png</x:v>
+        <x:v>members/teacher-006/avatar.png</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
         <x:v>teacher</x:v>
@@ -522,7 +543,7 @@
         <x:v>冯洋</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>avatar.jpg</x:v>
+        <x:v>members/teacher-007/avatar.jpg</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
         <x:v>teacher</x:v>
@@ -543,7 +564,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf3a3b9a234a4914"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa269498aaac4350"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -659,7 +680,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85c3b077d8174e31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab6d68befdac42dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -760,7 +781,255 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45664b52d52b40fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21341950a0454b83"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="27" customHeight="1">
+      <x:c r="A1" s="14" t="str">
+        <x:v>alias</x:v>
+      </x:c>
+      <x:c r="B1" s="14" t="str">
+        <x:v>member_id</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="26" customHeight="1">
+      <x:c r="A2" s="16" t="str">
+        <x:v>Zhenyu Chen</x:v>
+      </x:c>
+      <x:c r="B2" s="16" t="str">
+        <x:v>teacher-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="17" t="str">
+        <x:v>Chen Zhenyu</x:v>
+      </x:c>
+      <x:c r="B3" s="17" t="str">
+        <x:v>teacher-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="26" customHeight="1">
+      <x:c r="A4" s="17" t="str">
+        <x:v>Chunrong Fang</x:v>
+      </x:c>
+      <x:c r="B4" s="17" t="str">
+        <x:v>teacher-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26" customHeight="1">
+      <x:c r="A5" s="17" t="str">
+        <x:v>Fang Chunrong</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>teacher-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26" customHeight="1">
+      <x:c r="A6" s="17" t="str">
+        <x:v>Jia Liu</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>teacher-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26" customHeight="1">
+      <x:c r="A7" s="17" t="str">
+        <x:v>Liu Jia</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>teacher-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="26" customHeight="1">
+      <x:c r="A8" s="17" t="str">
+        <x:v>Tieke He</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>teacher-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26" customHeight="1">
+      <x:c r="A9" s="17" t="str">
+        <x:v>He Tieke</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>teacher-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="26" customHeight="1">
+      <x:c r="A10" s="17" t="str">
+        <x:v>Zhihong Zhao</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>teacher-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26" customHeight="1">
+      <x:c r="A11" s="17" t="str">
+        <x:v>Zhao Zhihong</x:v>
+      </x:c>
+      <x:c r="B11" s="17" t="str">
+        <x:v>teacher-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26" customHeight="1">
+      <x:c r="A12" s="17" t="str">
+        <x:v>Xingya Wang</x:v>
+      </x:c>
+      <x:c r="B12" s="17" t="str">
+        <x:v>teacher-006</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26" customHeight="1">
+      <x:c r="A13" s="17" t="str">
+        <x:v>Wang Xingya</x:v>
+      </x:c>
+      <x:c r="B13" s="17" t="str">
+        <x:v>teacher-006</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26" customHeight="1">
+      <x:c r="A14" s="17" t="str">
+        <x:v>Yang Feng</x:v>
+      </x:c>
+      <x:c r="B14" s="17" t="str">
+        <x:v>teacher-007</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="26" customHeight="1">
+      <x:c r="A15" s="17" t="str">
+        <x:v>Feng Yang</x:v>
+      </x:c>
+      <x:c r="B15" s="17" t="str">
+        <x:v>teacher-007</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="26" customHeight="1">
+      <x:c r="A16" s="17" t="str">
+        <x:v>An Guo</x:v>
+      </x:c>
+      <x:c r="B16" s="17" t="str">
+        <x:v>phd-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="26" customHeight="1">
+      <x:c r="A17" s="17" t="str">
+        <x:v>Guo An</x:v>
+      </x:c>
+      <x:c r="B17" s="17" t="str">
+        <x:v>phd-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="26" customHeight="1">
+      <x:c r="A18" s="17" t="str">
+        <x:v>Ruixiang Qian</x:v>
+      </x:c>
+      <x:c r="B18" s="17" t="str">
+        <x:v>phd-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="26" customHeight="1">
+      <x:c r="A19" s="17" t="str">
+        <x:v>Qian Ruixiang</x:v>
+      </x:c>
+      <x:c r="B19" s="17" t="str">
+        <x:v>phd-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="26" customHeight="1">
+      <x:c r="A20" s="17" t="str">
+        <x:v>Li Qiao</x:v>
+      </x:c>
+      <x:c r="B20" s="17" t="str">
+        <x:v>master-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="26" customHeight="1">
+      <x:c r="A21" s="17" t="str">
+        <x:v>Qiao Li</x:v>
+      </x:c>
+      <x:c r="B21" s="17" t="str">
+        <x:v>master-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="26" customHeight="1">
+      <x:c r="A22" s="17" t="str">
+        <x:v>Runxiang Rong</x:v>
+      </x:c>
+      <x:c r="B22" s="17" t="str">
+        <x:v>master-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="26" customHeight="1">
+      <x:c r="A23" s="17" t="str">
+        <x:v>Rong Runxiang</x:v>
+      </x:c>
+      <x:c r="B23" s="17" t="str">
+        <x:v>master-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="26" customHeight="1">
+      <x:c r="A24" s="17" t="str">
+        <x:v>Siqi Gu</x:v>
+      </x:c>
+      <x:c r="B24" s="17" t="str">
+        <x:v>phd-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="26" customHeight="1">
+      <x:c r="A25" s="17" t="str">
+        <x:v>Gu Siqi</x:v>
+      </x:c>
+      <x:c r="B25" s="17" t="str">
+        <x:v>phd-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="26" customHeight="1">
+      <x:c r="A26" s="17" t="str">
+        <x:v>Pin Ji</x:v>
+      </x:c>
+      <x:c r="B26" s="17" t="str">
+        <x:v>phd-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="26" customHeight="1">
+      <x:c r="A27" s="17" t="str">
+        <x:v>Ji Pin</x:v>
+      </x:c>
+      <x:c r="B27" s="17" t="str">
+        <x:v>phd-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="26" customHeight="1">
+      <x:c r="A28" s="17" t="str">
+        <x:v>Gaolei Yi</x:v>
+      </x:c>
+      <x:c r="B28" s="17" t="str">
+        <x:v>phd-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="26" customHeight="1">
+      <x:c r="A29" s="17" t="str">
+        <x:v>Yi Gaolei</x:v>
+      </x:c>
+      <x:c r="B29" s="17" t="str">
+        <x:v>phd-001</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6f7abbabb304cbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>